<commit_message>
fix(convert): apply ACU caps and record KB version
</commit_message>
<xml_diff>
--- a/docs/report-templates/samples/mapping-workbook.xlsx
+++ b/docs/report-templates/samples/mapping-workbook.xlsx
@@ -559,6 +559,11 @@
           <t>KB version</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">

</xml_diff>